<commit_message>
TODO SchemeRep paper (1/29/2024): * Make the 3-way ANOVA bar garph * Backburner: Look up the participation coefficient for the nodes in the t-modules * Individual differences between RSA x congruency response * Trial-by-trial link between RSA and congruency response * MVPA something?
</commit_message>
<xml_diff>
--- a/old/BNA_subregions.xlsx
+++ b/old/BNA_subregions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PycharmProjects_C\SchemeRep\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PycharmProjects_C\SchemeRep\old\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B87C2953-A84B-4EA9-8BCE-F1BA6A52747A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62E3B9B8-2538-4A55-BDC6-BE781FC90E41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="28110" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36650" yWindow="-870" windowWidth="23220" windowHeight="13890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1778,14 +1778,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2094,10 +2094,10 @@
       <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="6"/>
+      <c r="F1" s="4"/>
       <c r="G1" s="1" t="s">
         <v>529</v>
       </c>
@@ -2109,10 +2109,10 @@
       </c>
     </row>
     <row r="2" spans="1:9" ht="18" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -2124,10 +2124,10 @@
       <c r="E2" s="3">
         <v>2</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="5"/>
+      <c r="G2" s="6"/>
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
@@ -2136,8 +2136,8 @@
       </c>
     </row>
     <row r="3" spans="1:9" ht="18" customHeight="1">
-      <c r="A3" s="6"/>
-      <c r="B3" s="4"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
       <c r="C3" s="3" t="s">
         <v>12</v>
       </c>
@@ -2147,10 +2147,10 @@
       <c r="E3" s="3">
         <v>4</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>527</v>
       </c>
-      <c r="G3" s="5"/>
+      <c r="G3" s="6"/>
       <c r="H3" s="2" t="s">
         <v>13</v>
       </c>
@@ -2159,8 +2159,8 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="18" customHeight="1">
-      <c r="A4" s="6"/>
-      <c r="B4" s="4"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="3" t="s">
         <v>15</v>
       </c>
@@ -2170,10 +2170,10 @@
       <c r="E4" s="3">
         <v>6</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="5"/>
+      <c r="G4" s="6"/>
       <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
@@ -2182,8 +2182,8 @@
       </c>
     </row>
     <row r="5" spans="1:9" ht="18" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="4"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="5"/>
       <c r="C5" s="3" t="s">
         <v>19</v>
       </c>
@@ -2193,10 +2193,10 @@
       <c r="E5" s="3">
         <v>8</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="5"/>
+      <c r="G5" s="6"/>
       <c r="H5" s="2" t="s">
         <v>21</v>
       </c>
@@ -2205,8 +2205,8 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="18" customHeight="1">
-      <c r="A6" s="6"/>
-      <c r="B6" s="4"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="5"/>
       <c r="C6" s="3" t="s">
         <v>23</v>
       </c>
@@ -2216,10 +2216,10 @@
       <c r="E6" s="3">
         <v>10</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="5"/>
+      <c r="G6" s="6"/>
       <c r="H6" s="2" t="s">
         <v>25</v>
       </c>
@@ -2228,8 +2228,8 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="18" customHeight="1">
-      <c r="A7" s="6"/>
-      <c r="B7" s="4"/>
+      <c r="A7" s="4"/>
+      <c r="B7" s="5"/>
       <c r="C7" s="3" t="s">
         <v>27</v>
       </c>
@@ -2239,10 +2239,10 @@
       <c r="E7" s="3">
         <v>12</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="5"/>
+      <c r="G7" s="6"/>
       <c r="H7" s="2" t="s">
         <v>29</v>
       </c>
@@ -2251,8 +2251,8 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="18" customHeight="1">
-      <c r="A8" s="6"/>
-      <c r="B8" s="4"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="5"/>
       <c r="C8" s="3" t="s">
         <v>31</v>
       </c>
@@ -2262,10 +2262,10 @@
       <c r="E8" s="3">
         <v>14</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G8" s="5"/>
+      <c r="G8" s="6"/>
       <c r="H8" s="2" t="s">
         <v>33</v>
       </c>
@@ -2274,8 +2274,8 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="18" customHeight="1">
-      <c r="A9" s="6"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="4"/>
+      <c r="B9" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C9" s="3" t="s">
@@ -2287,10 +2287,10 @@
       <c r="E9" s="3">
         <v>16</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="G9" s="5"/>
+      <c r="G9" s="6"/>
       <c r="H9" s="2" t="s">
         <v>38</v>
       </c>
@@ -2299,8 +2299,8 @@
       </c>
     </row>
     <row r="10" spans="1:9" ht="18" customHeight="1">
-      <c r="A10" s="6"/>
-      <c r="B10" s="4"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="5"/>
       <c r="C10" s="3" t="s">
         <v>40</v>
       </c>
@@ -2310,10 +2310,10 @@
       <c r="E10" s="3">
         <v>18</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G10" s="5"/>
+      <c r="G10" s="6"/>
       <c r="H10" s="2" t="s">
         <v>42</v>
       </c>
@@ -2322,8 +2322,8 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="18" customHeight="1">
-      <c r="A11" s="6"/>
-      <c r="B11" s="4"/>
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
       <c r="C11" s="3" t="s">
         <v>44</v>
       </c>
@@ -2333,10 +2333,10 @@
       <c r="E11" s="3">
         <v>20</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="5"/>
+      <c r="G11" s="6"/>
       <c r="H11" s="2" t="s">
         <v>46</v>
       </c>
@@ -2345,8 +2345,8 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="18" customHeight="1">
-      <c r="A12" s="6"/>
-      <c r="B12" s="4"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="5"/>
       <c r="C12" s="3" t="s">
         <v>48</v>
       </c>
@@ -2356,10 +2356,10 @@
       <c r="E12" s="3">
         <v>22</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="G12" s="5"/>
+      <c r="G12" s="6"/>
       <c r="H12" s="2" t="s">
         <v>50</v>
       </c>
@@ -2368,8 +2368,8 @@
       </c>
     </row>
     <row r="13" spans="1:9" ht="18" customHeight="1">
-      <c r="A13" s="6"/>
-      <c r="B13" s="4"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="5"/>
       <c r="C13" s="3" t="s">
         <v>52</v>
       </c>
@@ -2379,10 +2379,10 @@
       <c r="E13" s="3">
         <v>24</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F13" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="G13" s="5"/>
+      <c r="G13" s="6"/>
       <c r="H13" s="2" t="s">
         <v>54</v>
       </c>
@@ -2391,8 +2391,8 @@
       </c>
     </row>
     <row r="14" spans="1:9" ht="18" customHeight="1">
-      <c r="A14" s="6"/>
-      <c r="B14" s="4"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="5"/>
       <c r="C14" s="3" t="s">
         <v>56</v>
       </c>
@@ -2402,10 +2402,10 @@
       <c r="E14" s="3">
         <v>26</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="5"/>
+      <c r="G14" s="6"/>
       <c r="H14" s="2" t="s">
         <v>58</v>
       </c>
@@ -2414,8 +2414,8 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="18" customHeight="1">
-      <c r="A15" s="6"/>
-      <c r="B15" s="4"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
       <c r="C15" s="3" t="s">
         <v>60</v>
       </c>
@@ -2425,10 +2425,10 @@
       <c r="E15" s="3">
         <v>28</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="G15" s="5"/>
+      <c r="G15" s="6"/>
       <c r="H15" s="2" t="s">
         <v>62</v>
       </c>
@@ -2437,8 +2437,8 @@
       </c>
     </row>
     <row r="16" spans="1:9" ht="18" customHeight="1">
-      <c r="A16" s="6"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="4"/>
+      <c r="B16" s="5" t="s">
         <v>64</v>
       </c>
       <c r="C16" s="3" t="s">
@@ -2450,10 +2450,10 @@
       <c r="E16" s="3">
         <v>30</v>
       </c>
-      <c r="F16" s="5" t="s">
+      <c r="F16" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="G16" s="5"/>
+      <c r="G16" s="6"/>
       <c r="H16" s="2" t="s">
         <v>67</v>
       </c>
@@ -2462,8 +2462,8 @@
       </c>
     </row>
     <row r="17" spans="1:9" ht="18" customHeight="1">
-      <c r="A17" s="6"/>
-      <c r="B17" s="4"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="5"/>
       <c r="C17" s="3" t="s">
         <v>69</v>
       </c>
@@ -2473,10 +2473,10 @@
       <c r="E17" s="3">
         <v>32</v>
       </c>
-      <c r="F17" s="5" t="s">
+      <c r="F17" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="G17" s="5"/>
+      <c r="G17" s="6"/>
       <c r="H17" s="2" t="s">
         <v>71</v>
       </c>
@@ -2485,8 +2485,8 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="18" customHeight="1">
-      <c r="A18" s="6"/>
-      <c r="B18" s="4"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="5"/>
       <c r="C18" s="3" t="s">
         <v>73</v>
       </c>
@@ -2496,10 +2496,10 @@
       <c r="E18" s="3">
         <v>34</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F18" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G18" s="5"/>
+      <c r="G18" s="6"/>
       <c r="H18" s="2" t="s">
         <v>75</v>
       </c>
@@ -2508,8 +2508,8 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="18" customHeight="1">
-      <c r="A19" s="6"/>
-      <c r="B19" s="4"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="5"/>
       <c r="C19" s="3" t="s">
         <v>77</v>
       </c>
@@ -2519,10 +2519,10 @@
       <c r="E19" s="3">
         <v>36</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="5"/>
+      <c r="G19" s="6"/>
       <c r="H19" s="2" t="s">
         <v>79</v>
       </c>
@@ -2531,8 +2531,8 @@
       </c>
     </row>
     <row r="20" spans="1:9" ht="18" customHeight="1">
-      <c r="A20" s="6"/>
-      <c r="B20" s="4"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="5"/>
       <c r="C20" s="3" t="s">
         <v>81</v>
       </c>
@@ -2542,10 +2542,10 @@
       <c r="E20" s="3">
         <v>38</v>
       </c>
-      <c r="F20" s="5" t="s">
+      <c r="F20" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="G20" s="5"/>
+      <c r="G20" s="6"/>
       <c r="H20" s="2" t="s">
         <v>83</v>
       </c>
@@ -2554,8 +2554,8 @@
       </c>
     </row>
     <row r="21" spans="1:9" ht="18" customHeight="1">
-      <c r="A21" s="6"/>
-      <c r="B21" s="4"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="5"/>
       <c r="C21" s="3" t="s">
         <v>85</v>
       </c>
@@ -2565,10 +2565,10 @@
       <c r="E21" s="3">
         <v>40</v>
       </c>
-      <c r="F21" s="5" t="s">
+      <c r="F21" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="G21" s="5"/>
+      <c r="G21" s="6"/>
       <c r="H21" s="2" t="s">
         <v>87</v>
       </c>
@@ -2577,8 +2577,8 @@
       </c>
     </row>
     <row r="22" spans="1:9" ht="18" customHeight="1">
-      <c r="A22" s="6"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="4"/>
+      <c r="B22" s="5" t="s">
         <v>89</v>
       </c>
       <c r="C22" s="3" t="s">
@@ -2590,10 +2590,10 @@
       <c r="E22" s="3">
         <v>42</v>
       </c>
-      <c r="F22" s="5" t="s">
+      <c r="F22" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="5"/>
+      <c r="G22" s="6"/>
       <c r="H22" s="2" t="s">
         <v>92</v>
       </c>
@@ -2602,8 +2602,8 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="18" customHeight="1">
-      <c r="A23" s="6"/>
-      <c r="B23" s="4"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="5"/>
       <c r="C23" s="3" t="s">
         <v>94</v>
       </c>
@@ -2613,10 +2613,10 @@
       <c r="E23" s="3">
         <v>44</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="G23" s="5"/>
+      <c r="G23" s="6"/>
       <c r="H23" s="2" t="s">
         <v>96</v>
       </c>
@@ -2625,8 +2625,8 @@
       </c>
     </row>
     <row r="24" spans="1:9" ht="18" customHeight="1">
-      <c r="A24" s="6"/>
-      <c r="B24" s="4"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="5"/>
       <c r="C24" s="3" t="s">
         <v>98</v>
       </c>
@@ -2636,10 +2636,10 @@
       <c r="E24" s="3">
         <v>46</v>
       </c>
-      <c r="F24" s="5" t="s">
+      <c r="F24" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="G24" s="5"/>
+      <c r="G24" s="6"/>
       <c r="H24" s="2" t="s">
         <v>100</v>
       </c>
@@ -2648,8 +2648,8 @@
       </c>
     </row>
     <row r="25" spans="1:9" ht="18" customHeight="1">
-      <c r="A25" s="6"/>
-      <c r="B25" s="4"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="5"/>
       <c r="C25" s="3" t="s">
         <v>102</v>
       </c>
@@ -2659,10 +2659,10 @@
       <c r="E25" s="3">
         <v>48</v>
       </c>
-      <c r="F25" s="5" t="s">
+      <c r="F25" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="G25" s="5"/>
+      <c r="G25" s="6"/>
       <c r="H25" s="2" t="s">
         <v>104</v>
       </c>
@@ -2671,8 +2671,8 @@
       </c>
     </row>
     <row r="26" spans="1:9" ht="18" customHeight="1">
-      <c r="A26" s="6"/>
-      <c r="B26" s="4"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="5"/>
       <c r="C26" s="3" t="s">
         <v>106</v>
       </c>
@@ -2682,10 +2682,10 @@
       <c r="E26" s="3">
         <v>50</v>
       </c>
-      <c r="F26" s="5" t="s">
+      <c r="F26" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="G26" s="5"/>
+      <c r="G26" s="6"/>
       <c r="H26" s="2" t="s">
         <v>108</v>
       </c>
@@ -2694,8 +2694,8 @@
       </c>
     </row>
     <row r="27" spans="1:9" ht="18" customHeight="1">
-      <c r="A27" s="6"/>
-      <c r="B27" s="4"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="5"/>
       <c r="C27" s="3" t="s">
         <v>110</v>
       </c>
@@ -2705,10 +2705,10 @@
       <c r="E27" s="3">
         <v>52</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="G27" s="5"/>
+      <c r="G27" s="6"/>
       <c r="H27" s="2" t="s">
         <v>112</v>
       </c>
@@ -2717,8 +2717,8 @@
       </c>
     </row>
     <row r="28" spans="1:9" ht="18" customHeight="1">
-      <c r="A28" s="6"/>
-      <c r="B28" s="4" t="s">
+      <c r="A28" s="4"/>
+      <c r="B28" s="5" t="s">
         <v>114</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -2730,10 +2730,10 @@
       <c r="E28" s="3">
         <v>54</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="G28" s="5"/>
+      <c r="G28" s="6"/>
       <c r="H28" s="2" t="s">
         <v>117</v>
       </c>
@@ -2742,8 +2742,8 @@
       </c>
     </row>
     <row r="29" spans="1:9" ht="18" customHeight="1">
-      <c r="A29" s="6"/>
-      <c r="B29" s="4"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="5"/>
       <c r="C29" s="3" t="s">
         <v>119</v>
       </c>
@@ -2753,10 +2753,10 @@
       <c r="E29" s="3">
         <v>56</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F29" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="G29" s="5"/>
+      <c r="G29" s="6"/>
       <c r="H29" s="2" t="s">
         <v>121</v>
       </c>
@@ -2765,8 +2765,8 @@
       </c>
     </row>
     <row r="30" spans="1:9" ht="18" customHeight="1">
-      <c r="A30" s="6"/>
-      <c r="B30" s="4"/>
+      <c r="A30" s="4"/>
+      <c r="B30" s="5"/>
       <c r="C30" s="3" t="s">
         <v>123</v>
       </c>
@@ -2776,10 +2776,10 @@
       <c r="E30" s="3">
         <v>58</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="G30" s="5"/>
+      <c r="G30" s="6"/>
       <c r="H30" s="2" t="s">
         <v>125</v>
       </c>
@@ -2788,8 +2788,8 @@
       </c>
     </row>
     <row r="31" spans="1:9" ht="18" customHeight="1">
-      <c r="A31" s="6"/>
-      <c r="B31" s="4"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="5"/>
       <c r="C31" s="3" t="s">
         <v>127</v>
       </c>
@@ -2799,10 +2799,10 @@
       <c r="E31" s="3">
         <v>60</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="G31" s="5"/>
+      <c r="G31" s="6"/>
       <c r="H31" s="2" t="s">
         <v>129</v>
       </c>
@@ -2811,8 +2811,8 @@
       </c>
     </row>
     <row r="32" spans="1:9" ht="18" customHeight="1">
-      <c r="A32" s="6"/>
-      <c r="B32" s="4"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="5"/>
       <c r="C32" s="3" t="s">
         <v>131</v>
       </c>
@@ -2822,10 +2822,10 @@
       <c r="E32" s="3">
         <v>62</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="F32" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="G32" s="5"/>
+      <c r="G32" s="6"/>
       <c r="H32" s="2" t="s">
         <v>133</v>
       </c>
@@ -2834,8 +2834,8 @@
       </c>
     </row>
     <row r="33" spans="1:9" ht="18" customHeight="1">
-      <c r="A33" s="6"/>
-      <c r="B33" s="4"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="5"/>
       <c r="C33" s="3" t="s">
         <v>135</v>
       </c>
@@ -2845,10 +2845,10 @@
       <c r="E33" s="3">
         <v>64</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="G33" s="5"/>
+      <c r="G33" s="6"/>
       <c r="H33" s="2" t="s">
         <v>137</v>
       </c>
@@ -2857,8 +2857,8 @@
       </c>
     </row>
     <row r="34" spans="1:9" ht="18" customHeight="1">
-      <c r="A34" s="6"/>
-      <c r="B34" s="4" t="s">
+      <c r="A34" s="4"/>
+      <c r="B34" s="5" t="s">
         <v>139</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -2870,10 +2870,10 @@
       <c r="E34" s="3">
         <v>66</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="G34" s="5"/>
+      <c r="G34" s="6"/>
       <c r="H34" s="2" t="s">
         <v>142</v>
       </c>
@@ -2882,8 +2882,8 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="18" customHeight="1">
-      <c r="A35" s="6"/>
-      <c r="B35" s="4"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="5"/>
       <c r="C35" s="3" t="s">
         <v>144</v>
       </c>
@@ -2893,10 +2893,10 @@
       <c r="E35" s="3">
         <v>68</v>
       </c>
-      <c r="F35" s="5" t="s">
+      <c r="F35" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="G35" s="5"/>
+      <c r="G35" s="6"/>
       <c r="H35" s="2" t="s">
         <v>146</v>
       </c>
@@ -2905,10 +2905,10 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="18" customHeight="1">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="B36" s="4" t="s">
+      <c r="B36" s="5" t="s">
         <v>149</v>
       </c>
       <c r="C36" s="3" t="s">
@@ -2920,10 +2920,10 @@
       <c r="E36" s="3">
         <v>70</v>
       </c>
-      <c r="F36" s="5" t="s">
+      <c r="F36" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="G36" s="5"/>
+      <c r="G36" s="6"/>
       <c r="H36" s="2" t="s">
         <v>152</v>
       </c>
@@ -2932,8 +2932,8 @@
       </c>
     </row>
     <row r="37" spans="1:9" ht="18" customHeight="1">
-      <c r="A37" s="6"/>
-      <c r="B37" s="4"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="5"/>
       <c r="C37" s="3" t="s">
         <v>154</v>
       </c>
@@ -2943,10 +2943,10 @@
       <c r="E37" s="3">
         <v>72</v>
       </c>
-      <c r="F37" s="5" t="s">
+      <c r="F37" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="G37" s="5"/>
+      <c r="G37" s="6"/>
       <c r="H37" s="2" t="s">
         <v>156</v>
       </c>
@@ -2955,8 +2955,8 @@
       </c>
     </row>
     <row r="38" spans="1:9" ht="18" customHeight="1">
-      <c r="A38" s="6"/>
-      <c r="B38" s="4"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="5"/>
       <c r="C38" s="3" t="s">
         <v>158</v>
       </c>
@@ -2966,10 +2966,10 @@
       <c r="E38" s="3">
         <v>74</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="F38" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="G38" s="5"/>
+      <c r="G38" s="6"/>
       <c r="H38" s="2" t="s">
         <v>160</v>
       </c>
@@ -2978,8 +2978,8 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="18" customHeight="1">
-      <c r="A39" s="6"/>
-      <c r="B39" s="4"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="5"/>
       <c r="C39" s="3" t="s">
         <v>162</v>
       </c>
@@ -2989,10 +2989,10 @@
       <c r="E39" s="3">
         <v>76</v>
       </c>
-      <c r="F39" s="5" t="s">
+      <c r="F39" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="G39" s="5"/>
+      <c r="G39" s="6"/>
       <c r="H39" s="2" t="s">
         <v>164</v>
       </c>
@@ -3001,8 +3001,8 @@
       </c>
     </row>
     <row r="40" spans="1:9" ht="18" customHeight="1">
-      <c r="A40" s="6"/>
-      <c r="B40" s="4"/>
+      <c r="A40" s="4"/>
+      <c r="B40" s="5"/>
       <c r="C40" s="3" t="s">
         <v>166</v>
       </c>
@@ -3012,10 +3012,10 @@
       <c r="E40" s="3">
         <v>78</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="G40" s="5"/>
+      <c r="G40" s="6"/>
       <c r="H40" s="2" t="s">
         <v>168</v>
       </c>
@@ -3024,8 +3024,8 @@
       </c>
     </row>
     <row r="41" spans="1:9" ht="18" customHeight="1">
-      <c r="A41" s="6"/>
-      <c r="B41" s="4"/>
+      <c r="A41" s="4"/>
+      <c r="B41" s="5"/>
       <c r="C41" s="3" t="s">
         <v>170</v>
       </c>
@@ -3035,10 +3035,10 @@
       <c r="E41" s="3">
         <v>80</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="G41" s="5"/>
+      <c r="G41" s="6"/>
       <c r="H41" s="2" t="s">
         <v>172</v>
       </c>
@@ -3047,8 +3047,8 @@
       </c>
     </row>
     <row r="42" spans="1:9" ht="18" customHeight="1">
-      <c r="A42" s="6"/>
-      <c r="B42" s="4" t="s">
+      <c r="A42" s="4"/>
+      <c r="B42" s="5" t="s">
         <v>174</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -3060,10 +3060,10 @@
       <c r="E42" s="3">
         <v>82</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="F42" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="G42" s="5"/>
+      <c r="G42" s="6"/>
       <c r="H42" s="2" t="s">
         <v>177</v>
       </c>
@@ -3072,8 +3072,8 @@
       </c>
     </row>
     <row r="43" spans="1:9" ht="18" customHeight="1">
-      <c r="A43" s="6"/>
-      <c r="B43" s="4"/>
+      <c r="A43" s="4"/>
+      <c r="B43" s="5"/>
       <c r="C43" s="3" t="s">
         <v>179</v>
       </c>
@@ -3083,10 +3083,10 @@
       <c r="E43" s="3">
         <v>84</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="G43" s="5"/>
+      <c r="G43" s="6"/>
       <c r="H43" s="2" t="s">
         <v>181</v>
       </c>
@@ -3095,8 +3095,8 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="18" customHeight="1">
-      <c r="A44" s="6"/>
-      <c r="B44" s="4"/>
+      <c r="A44" s="4"/>
+      <c r="B44" s="5"/>
       <c r="C44" s="3" t="s">
         <v>183</v>
       </c>
@@ -3106,10 +3106,10 @@
       <c r="E44" s="3">
         <v>86</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="G44" s="5"/>
+      <c r="G44" s="6"/>
       <c r="H44" s="2" t="s">
         <v>185</v>
       </c>
@@ -3118,8 +3118,8 @@
       </c>
     </row>
     <row r="45" spans="1:9" ht="18" customHeight="1">
-      <c r="A45" s="6"/>
-      <c r="B45" s="4"/>
+      <c r="A45" s="4"/>
+      <c r="B45" s="5"/>
       <c r="C45" s="3" t="s">
         <v>187</v>
       </c>
@@ -3129,10 +3129,10 @@
       <c r="E45" s="3">
         <v>88</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="G45" s="5"/>
+      <c r="G45" s="6"/>
       <c r="H45" s="2" t="s">
         <v>189</v>
       </c>
@@ -3141,8 +3141,8 @@
       </c>
     </row>
     <row r="46" spans="1:9" ht="18" customHeight="1">
-      <c r="A46" s="6"/>
-      <c r="B46" s="4" t="s">
+      <c r="A46" s="4"/>
+      <c r="B46" s="5" t="s">
         <v>191</v>
       </c>
       <c r="C46" s="3" t="s">
@@ -3154,10 +3154,10 @@
       <c r="E46" s="3">
         <v>90</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="G46" s="5"/>
+      <c r="G46" s="6"/>
       <c r="H46" s="2" t="s">
         <v>194</v>
       </c>
@@ -3166,8 +3166,8 @@
       </c>
     </row>
     <row r="47" spans="1:9" ht="18" customHeight="1">
-      <c r="A47" s="6"/>
-      <c r="B47" s="4"/>
+      <c r="A47" s="4"/>
+      <c r="B47" s="5"/>
       <c r="C47" s="3" t="s">
         <v>196</v>
       </c>
@@ -3177,10 +3177,10 @@
       <c r="E47" s="3">
         <v>92</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="F47" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="G47" s="5"/>
+      <c r="G47" s="6"/>
       <c r="H47" s="2" t="s">
         <v>198</v>
       </c>
@@ -3189,8 +3189,8 @@
       </c>
     </row>
     <row r="48" spans="1:9" ht="18" customHeight="1">
-      <c r="A48" s="6"/>
-      <c r="B48" s="4"/>
+      <c r="A48" s="4"/>
+      <c r="B48" s="5"/>
       <c r="C48" s="3" t="s">
         <v>200</v>
       </c>
@@ -3200,10 +3200,10 @@
       <c r="E48" s="3">
         <v>94</v>
       </c>
-      <c r="F48" s="5" t="s">
+      <c r="F48" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="G48" s="5"/>
+      <c r="G48" s="6"/>
       <c r="H48" s="2" t="s">
         <v>202</v>
       </c>
@@ -3212,8 +3212,8 @@
       </c>
     </row>
     <row r="49" spans="1:9" ht="18" customHeight="1">
-      <c r="A49" s="6"/>
-      <c r="B49" s="4"/>
+      <c r="A49" s="4"/>
+      <c r="B49" s="5"/>
       <c r="C49" s="3" t="s">
         <v>204</v>
       </c>
@@ -3223,10 +3223,10 @@
       <c r="E49" s="3">
         <v>96</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="G49" s="5"/>
+      <c r="G49" s="6"/>
       <c r="H49" s="2" t="s">
         <v>206</v>
       </c>
@@ -3235,8 +3235,8 @@
       </c>
     </row>
     <row r="50" spans="1:9" ht="18" customHeight="1">
-      <c r="A50" s="6"/>
-      <c r="B50" s="4"/>
+      <c r="A50" s="4"/>
+      <c r="B50" s="5"/>
       <c r="C50" s="3" t="s">
         <v>208</v>
       </c>
@@ -3246,10 +3246,10 @@
       <c r="E50" s="3">
         <v>98</v>
       </c>
-      <c r="F50" s="5" t="s">
+      <c r="F50" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="G50" s="5"/>
+      <c r="G50" s="6"/>
       <c r="H50" s="2" t="s">
         <v>210</v>
       </c>
@@ -3258,8 +3258,8 @@
       </c>
     </row>
     <row r="51" spans="1:9" ht="18" customHeight="1">
-      <c r="A51" s="6"/>
-      <c r="B51" s="4"/>
+      <c r="A51" s="4"/>
+      <c r="B51" s="5"/>
       <c r="C51" s="3" t="s">
         <v>212</v>
       </c>
@@ -3269,10 +3269,10 @@
       <c r="E51" s="3">
         <v>100</v>
       </c>
-      <c r="F51" s="5" t="s">
+      <c r="F51" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="G51" s="5"/>
+      <c r="G51" s="6"/>
       <c r="H51" s="2" t="s">
         <v>214</v>
       </c>
@@ -3281,8 +3281,8 @@
       </c>
     </row>
     <row r="52" spans="1:9" ht="18" customHeight="1">
-      <c r="A52" s="6"/>
-      <c r="B52" s="4"/>
+      <c r="A52" s="4"/>
+      <c r="B52" s="5"/>
       <c r="C52" s="3" t="s">
         <v>216</v>
       </c>
@@ -3292,10 +3292,10 @@
       <c r="E52" s="3">
         <v>102</v>
       </c>
-      <c r="F52" s="5" t="s">
+      <c r="F52" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="G52" s="5"/>
+      <c r="G52" s="6"/>
       <c r="H52" s="2" t="s">
         <v>218</v>
       </c>
@@ -3304,8 +3304,8 @@
       </c>
     </row>
     <row r="53" spans="1:9" ht="18" customHeight="1">
-      <c r="A53" s="6"/>
-      <c r="B53" s="4" t="s">
+      <c r="A53" s="4"/>
+      <c r="B53" s="5" t="s">
         <v>220</v>
       </c>
       <c r="C53" s="3" t="s">
@@ -3317,10 +3317,10 @@
       <c r="E53" s="3">
         <v>104</v>
       </c>
-      <c r="F53" s="5" t="s">
+      <c r="F53" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="G53" s="5"/>
+      <c r="G53" s="6"/>
       <c r="H53" s="2" t="s">
         <v>223</v>
       </c>
@@ -3329,8 +3329,8 @@
       </c>
     </row>
     <row r="54" spans="1:9" ht="18" customHeight="1">
-      <c r="A54" s="6"/>
-      <c r="B54" s="4"/>
+      <c r="A54" s="4"/>
+      <c r="B54" s="5"/>
       <c r="C54" s="3" t="s">
         <v>225</v>
       </c>
@@ -3340,10 +3340,10 @@
       <c r="E54" s="3">
         <v>106</v>
       </c>
-      <c r="F54" s="5" t="s">
+      <c r="F54" s="6" t="s">
         <v>226</v>
       </c>
-      <c r="G54" s="5"/>
+      <c r="G54" s="6"/>
       <c r="H54" s="2" t="s">
         <v>227</v>
       </c>
@@ -3352,8 +3352,8 @@
       </c>
     </row>
     <row r="55" spans="1:9" ht="18" customHeight="1">
-      <c r="A55" s="6"/>
-      <c r="B55" s="4"/>
+      <c r="A55" s="4"/>
+      <c r="B55" s="5"/>
       <c r="C55" s="3" t="s">
         <v>229</v>
       </c>
@@ -3363,10 +3363,10 @@
       <c r="E55" s="3">
         <v>108</v>
       </c>
-      <c r="F55" s="5" t="s">
+      <c r="F55" s="6" t="s">
         <v>230</v>
       </c>
-      <c r="G55" s="5"/>
+      <c r="G55" s="6"/>
       <c r="H55" s="2" t="s">
         <v>231</v>
       </c>
@@ -3375,8 +3375,8 @@
       </c>
     </row>
     <row r="56" spans="1:9" ht="18" customHeight="1">
-      <c r="A56" s="6"/>
-      <c r="B56" s="4" t="s">
+      <c r="A56" s="4"/>
+      <c r="B56" s="5" t="s">
         <v>233</v>
       </c>
       <c r="C56" s="3" t="s">
@@ -3388,10 +3388,10 @@
       <c r="E56" s="3">
         <v>110</v>
       </c>
-      <c r="F56" s="5" t="s">
+      <c r="F56" s="6" t="s">
         <v>235</v>
       </c>
-      <c r="G56" s="5"/>
+      <c r="G56" s="6"/>
       <c r="H56" s="2" t="s">
         <v>236</v>
       </c>
@@ -3400,8 +3400,8 @@
       </c>
     </row>
     <row r="57" spans="1:9" ht="18" customHeight="1">
-      <c r="A57" s="6"/>
-      <c r="B57" s="4"/>
+      <c r="A57" s="4"/>
+      <c r="B57" s="5"/>
       <c r="C57" s="3" t="s">
         <v>238</v>
       </c>
@@ -3411,10 +3411,10 @@
       <c r="E57" s="3">
         <v>112</v>
       </c>
-      <c r="F57" s="5" t="s">
+      <c r="F57" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="G57" s="5"/>
+      <c r="G57" s="6"/>
       <c r="H57" s="2" t="s">
         <v>240</v>
       </c>
@@ -3423,8 +3423,8 @@
       </c>
     </row>
     <row r="58" spans="1:9" ht="18" customHeight="1">
-      <c r="A58" s="6"/>
-      <c r="B58" s="4"/>
+      <c r="A58" s="4"/>
+      <c r="B58" s="5"/>
       <c r="C58" s="3" t="s">
         <v>242</v>
       </c>
@@ -3434,10 +3434,10 @@
       <c r="E58" s="3">
         <v>114</v>
       </c>
-      <c r="F58" s="5" t="s">
+      <c r="F58" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="G58" s="5"/>
+      <c r="G58" s="6"/>
       <c r="H58" s="2" t="s">
         <v>244</v>
       </c>
@@ -3446,8 +3446,8 @@
       </c>
     </row>
     <row r="59" spans="1:9" ht="18" customHeight="1">
-      <c r="A59" s="6"/>
-      <c r="B59" s="4"/>
+      <c r="A59" s="4"/>
+      <c r="B59" s="5"/>
       <c r="C59" s="3" t="s">
         <v>246</v>
       </c>
@@ -3457,10 +3457,10 @@
       <c r="E59" s="3">
         <v>116</v>
       </c>
-      <c r="F59" s="5" t="s">
+      <c r="F59" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="G59" s="5"/>
+      <c r="G59" s="6"/>
       <c r="H59" s="2" t="s">
         <v>248</v>
       </c>
@@ -3469,8 +3469,8 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="18" customHeight="1">
-      <c r="A60" s="6"/>
-      <c r="B60" s="4"/>
+      <c r="A60" s="4"/>
+      <c r="B60" s="5"/>
       <c r="C60" s="3" t="s">
         <v>250</v>
       </c>
@@ -3480,10 +3480,10 @@
       <c r="E60" s="3">
         <v>118</v>
       </c>
-      <c r="F60" s="5" t="s">
+      <c r="F60" s="6" t="s">
         <v>251</v>
       </c>
-      <c r="G60" s="5"/>
+      <c r="G60" s="6"/>
       <c r="H60" s="2" t="s">
         <v>252</v>
       </c>
@@ -3492,8 +3492,8 @@
       </c>
     </row>
     <row r="61" spans="1:9" ht="18" customHeight="1">
-      <c r="A61" s="6"/>
-      <c r="B61" s="4"/>
+      <c r="A61" s="4"/>
+      <c r="B61" s="5"/>
       <c r="C61" s="3" t="s">
         <v>254</v>
       </c>
@@ -3503,10 +3503,10 @@
       <c r="E61" s="3">
         <v>120</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="F61" s="6" t="s">
         <v>255</v>
       </c>
-      <c r="G61" s="5"/>
+      <c r="G61" s="6"/>
       <c r="H61" s="2" t="s">
         <v>256</v>
       </c>
@@ -3515,8 +3515,8 @@
       </c>
     </row>
     <row r="62" spans="1:9" ht="18" customHeight="1">
-      <c r="A62" s="6"/>
-      <c r="B62" s="4" t="s">
+      <c r="A62" s="4"/>
+      <c r="B62" s="5" t="s">
         <v>258</v>
       </c>
       <c r="C62" s="3" t="s">
@@ -3528,10 +3528,10 @@
       <c r="E62" s="3">
         <v>122</v>
       </c>
-      <c r="F62" s="5" t="s">
+      <c r="F62" s="6" t="s">
         <v>260</v>
       </c>
-      <c r="G62" s="5"/>
+      <c r="G62" s="6"/>
       <c r="H62" s="2" t="s">
         <v>261</v>
       </c>
@@ -3540,8 +3540,8 @@
       </c>
     </row>
     <row r="63" spans="1:9" ht="18" customHeight="1">
-      <c r="A63" s="6"/>
-      <c r="B63" s="4"/>
+      <c r="A63" s="4"/>
+      <c r="B63" s="5"/>
       <c r="C63" s="3" t="s">
         <v>263</v>
       </c>
@@ -3551,10 +3551,10 @@
       <c r="E63" s="3">
         <v>124</v>
       </c>
-      <c r="F63" s="5" t="s">
+      <c r="F63" s="6" t="s">
         <v>530</v>
       </c>
-      <c r="G63" s="5"/>
+      <c r="G63" s="6"/>
       <c r="H63" s="2" t="s">
         <v>264</v>
       </c>
@@ -3563,10 +3563,10 @@
       </c>
     </row>
     <row r="64" spans="1:9" ht="18" customHeight="1">
-      <c r="A64" s="6" t="s">
+      <c r="A64" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="B64" s="4" t="s">
+      <c r="B64" s="5" t="s">
         <v>267</v>
       </c>
       <c r="C64" s="3" t="s">
@@ -3578,10 +3578,10 @@
       <c r="E64" s="3">
         <v>126</v>
       </c>
-      <c r="F64" s="5" t="s">
+      <c r="F64" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="G64" s="5"/>
+      <c r="G64" s="6"/>
       <c r="H64" s="2" t="s">
         <v>270</v>
       </c>
@@ -3590,8 +3590,8 @@
       </c>
     </row>
     <row r="65" spans="1:9" ht="18" customHeight="1">
-      <c r="A65" s="6"/>
-      <c r="B65" s="4"/>
+      <c r="A65" s="4"/>
+      <c r="B65" s="5"/>
       <c r="C65" s="3" t="s">
         <v>272</v>
       </c>
@@ -3601,10 +3601,10 @@
       <c r="E65" s="3">
         <v>128</v>
       </c>
-      <c r="F65" s="5" t="s">
+      <c r="F65" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="G65" s="5"/>
+      <c r="G65" s="6"/>
       <c r="H65" s="2" t="s">
         <v>274</v>
       </c>
@@ -3613,8 +3613,8 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="18" customHeight="1">
-      <c r="A66" s="6"/>
-      <c r="B66" s="4"/>
+      <c r="A66" s="4"/>
+      <c r="B66" s="5"/>
       <c r="C66" s="3" t="s">
         <v>276</v>
       </c>
@@ -3624,10 +3624,10 @@
       <c r="E66" s="3">
         <v>130</v>
       </c>
-      <c r="F66" s="5" t="s">
+      <c r="F66" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="G66" s="5"/>
+      <c r="G66" s="6"/>
       <c r="H66" s="2" t="s">
         <v>278</v>
       </c>
@@ -3636,8 +3636,8 @@
       </c>
     </row>
     <row r="67" spans="1:9" ht="18" customHeight="1">
-      <c r="A67" s="6"/>
-      <c r="B67" s="4"/>
+      <c r="A67" s="4"/>
+      <c r="B67" s="5"/>
       <c r="C67" s="3" t="s">
         <v>280</v>
       </c>
@@ -3647,10 +3647,10 @@
       <c r="E67" s="3">
         <v>132</v>
       </c>
-      <c r="F67" s="5" t="s">
+      <c r="F67" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="G67" s="5"/>
+      <c r="G67" s="6"/>
       <c r="H67" s="2" t="s">
         <v>282</v>
       </c>
@@ -3659,8 +3659,8 @@
       </c>
     </row>
     <row r="68" spans="1:9" ht="18" customHeight="1">
-      <c r="A68" s="6"/>
-      <c r="B68" s="4"/>
+      <c r="A68" s="4"/>
+      <c r="B68" s="5"/>
       <c r="C68" s="3" t="s">
         <v>284</v>
       </c>
@@ -3670,10 +3670,10 @@
       <c r="E68" s="3">
         <v>134</v>
       </c>
-      <c r="F68" s="5" t="s">
+      <c r="F68" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="G68" s="5"/>
+      <c r="G68" s="6"/>
       <c r="H68" s="2" t="s">
         <v>286</v>
       </c>
@@ -3682,8 +3682,8 @@
       </c>
     </row>
     <row r="69" spans="1:9" ht="18" customHeight="1">
-      <c r="A69" s="6"/>
-      <c r="B69" s="4" t="s">
+      <c r="A69" s="4"/>
+      <c r="B69" s="5" t="s">
         <v>288</v>
       </c>
       <c r="C69" s="3" t="s">
@@ -3695,10 +3695,10 @@
       <c r="E69" s="3">
         <v>136</v>
       </c>
-      <c r="F69" s="5" t="s">
+      <c r="F69" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="G69" s="5"/>
+      <c r="G69" s="6"/>
       <c r="H69" s="2" t="s">
         <v>291</v>
       </c>
@@ -3707,8 +3707,8 @@
       </c>
     </row>
     <row r="70" spans="1:9" ht="18" customHeight="1">
-      <c r="A70" s="6"/>
-      <c r="B70" s="4"/>
+      <c r="A70" s="4"/>
+      <c r="B70" s="5"/>
       <c r="C70" s="3" t="s">
         <v>293</v>
       </c>
@@ -3718,10 +3718,10 @@
       <c r="E70" s="3">
         <v>138</v>
       </c>
-      <c r="F70" s="5" t="s">
+      <c r="F70" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="G70" s="5"/>
+      <c r="G70" s="6"/>
       <c r="H70" s="2" t="s">
         <v>295</v>
       </c>
@@ -3730,8 +3730,8 @@
       </c>
     </row>
     <row r="71" spans="1:9" ht="18" customHeight="1">
-      <c r="A71" s="6"/>
-      <c r="B71" s="4"/>
+      <c r="A71" s="4"/>
+      <c r="B71" s="5"/>
       <c r="C71" s="3" t="s">
         <v>297</v>
       </c>
@@ -3741,10 +3741,10 @@
       <c r="E71" s="3">
         <v>140</v>
       </c>
-      <c r="F71" s="5" t="s">
+      <c r="F71" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="G71" s="5"/>
+      <c r="G71" s="6"/>
       <c r="H71" s="2" t="s">
         <v>299</v>
       </c>
@@ -3753,8 +3753,8 @@
       </c>
     </row>
     <row r="72" spans="1:9" ht="18" customHeight="1">
-      <c r="A72" s="6"/>
-      <c r="B72" s="4"/>
+      <c r="A72" s="4"/>
+      <c r="B72" s="5"/>
       <c r="C72" s="3" t="s">
         <v>301</v>
       </c>
@@ -3764,10 +3764,10 @@
       <c r="E72" s="3">
         <v>142</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="F72" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="G72" s="5"/>
+      <c r="G72" s="6"/>
       <c r="H72" s="2" t="s">
         <v>303</v>
       </c>
@@ -3776,8 +3776,8 @@
       </c>
     </row>
     <row r="73" spans="1:9" ht="18" customHeight="1">
-      <c r="A73" s="6"/>
-      <c r="B73" s="4"/>
+      <c r="A73" s="4"/>
+      <c r="B73" s="5"/>
       <c r="C73" s="3" t="s">
         <v>305</v>
       </c>
@@ -3787,10 +3787,10 @@
       <c r="E73" s="3">
         <v>144</v>
       </c>
-      <c r="F73" s="5" t="s">
+      <c r="F73" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="G73" s="5"/>
+      <c r="G73" s="6"/>
       <c r="H73" s="2" t="s">
         <v>307</v>
       </c>
@@ -3799,8 +3799,8 @@
       </c>
     </row>
     <row r="74" spans="1:9" ht="18" customHeight="1">
-      <c r="A74" s="6"/>
-      <c r="B74" s="4"/>
+      <c r="A74" s="4"/>
+      <c r="B74" s="5"/>
       <c r="C74" s="3" t="s">
         <v>309</v>
       </c>
@@ -3810,10 +3810,10 @@
       <c r="E74" s="3">
         <v>146</v>
       </c>
-      <c r="F74" s="5" t="s">
+      <c r="F74" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="G74" s="5"/>
+      <c r="G74" s="6"/>
       <c r="H74" s="2" t="s">
         <v>311</v>
       </c>
@@ -3822,8 +3822,8 @@
       </c>
     </row>
     <row r="75" spans="1:9" ht="18" customHeight="1">
-      <c r="A75" s="6"/>
-      <c r="B75" s="4" t="s">
+      <c r="A75" s="4"/>
+      <c r="B75" s="5" t="s">
         <v>313</v>
       </c>
       <c r="C75" s="3" t="s">
@@ -3835,10 +3835,10 @@
       <c r="E75" s="3">
         <v>148</v>
       </c>
-      <c r="F75" s="5" t="s">
+      <c r="F75" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="G75" s="5"/>
+      <c r="G75" s="6"/>
       <c r="H75" s="2" t="s">
         <v>316</v>
       </c>
@@ -3847,8 +3847,8 @@
       </c>
     </row>
     <row r="76" spans="1:9" ht="18" customHeight="1">
-      <c r="A76" s="6"/>
-      <c r="B76" s="4"/>
+      <c r="A76" s="4"/>
+      <c r="B76" s="5"/>
       <c r="C76" s="3" t="s">
         <v>318</v>
       </c>
@@ -3858,10 +3858,10 @@
       <c r="E76" s="3">
         <v>150</v>
       </c>
-      <c r="F76" s="5" t="s">
+      <c r="F76" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="G76" s="5"/>
+      <c r="G76" s="6"/>
       <c r="H76" s="2" t="s">
         <v>320</v>
       </c>
@@ -3870,8 +3870,8 @@
       </c>
     </row>
     <row r="77" spans="1:9" ht="18" customHeight="1">
-      <c r="A77" s="6"/>
-      <c r="B77" s="4"/>
+      <c r="A77" s="4"/>
+      <c r="B77" s="5"/>
       <c r="C77" s="3" t="s">
         <v>322</v>
       </c>
@@ -3881,10 +3881,10 @@
       <c r="E77" s="3">
         <v>152</v>
       </c>
-      <c r="F77" s="5" t="s">
+      <c r="F77" s="6" t="s">
         <v>323</v>
       </c>
-      <c r="G77" s="5"/>
+      <c r="G77" s="6"/>
       <c r="H77" s="2" t="s">
         <v>324</v>
       </c>
@@ -3893,8 +3893,8 @@
       </c>
     </row>
     <row r="78" spans="1:9" ht="18" customHeight="1">
-      <c r="A78" s="6"/>
-      <c r="B78" s="4"/>
+      <c r="A78" s="4"/>
+      <c r="B78" s="5"/>
       <c r="C78" s="3" t="s">
         <v>326</v>
       </c>
@@ -3904,10 +3904,10 @@
       <c r="E78" s="3">
         <v>154</v>
       </c>
-      <c r="F78" s="5" t="s">
+      <c r="F78" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="G78" s="5"/>
+      <c r="G78" s="6"/>
       <c r="H78" s="2" t="s">
         <v>328</v>
       </c>
@@ -3916,8 +3916,8 @@
       </c>
     </row>
     <row r="79" spans="1:9" ht="18" customHeight="1">
-      <c r="A79" s="6"/>
-      <c r="B79" s="4" t="s">
+      <c r="A79" s="4"/>
+      <c r="B79" s="5" t="s">
         <v>330</v>
       </c>
       <c r="C79" s="3" t="s">
@@ -3929,10 +3929,10 @@
       <c r="E79" s="3">
         <v>156</v>
       </c>
-      <c r="F79" s="5" t="s">
+      <c r="F79" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="G79" s="5"/>
+      <c r="G79" s="6"/>
       <c r="H79" s="2" t="s">
         <v>333</v>
       </c>
@@ -3941,8 +3941,8 @@
       </c>
     </row>
     <row r="80" spans="1:9" ht="18" customHeight="1">
-      <c r="A80" s="6"/>
-      <c r="B80" s="4"/>
+      <c r="A80" s="4"/>
+      <c r="B80" s="5"/>
       <c r="C80" s="3" t="s">
         <v>335</v>
       </c>
@@ -3952,10 +3952,10 @@
       <c r="E80" s="3">
         <v>158</v>
       </c>
-      <c r="F80" s="5" t="s">
+      <c r="F80" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="G80" s="5"/>
+      <c r="G80" s="6"/>
       <c r="H80" s="2" t="s">
         <v>337</v>
       </c>
@@ -3964,8 +3964,8 @@
       </c>
     </row>
     <row r="81" spans="1:9" ht="18" customHeight="1">
-      <c r="A81" s="6"/>
-      <c r="B81" s="4"/>
+      <c r="A81" s="4"/>
+      <c r="B81" s="5"/>
       <c r="C81" s="3" t="s">
         <v>339</v>
       </c>
@@ -3975,10 +3975,10 @@
       <c r="E81" s="3">
         <v>160</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="F81" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="G81" s="5"/>
+      <c r="G81" s="6"/>
       <c r="H81" s="2" t="s">
         <v>341</v>
       </c>
@@ -3987,8 +3987,8 @@
       </c>
     </row>
     <row r="82" spans="1:9" ht="18" customHeight="1">
-      <c r="A82" s="6"/>
-      <c r="B82" s="4"/>
+      <c r="A82" s="4"/>
+      <c r="B82" s="5"/>
       <c r="C82" s="3" t="s">
         <v>343</v>
       </c>
@@ -3998,10 +3998,10 @@
       <c r="E82" s="3">
         <v>162</v>
       </c>
-      <c r="F82" s="5" t="s">
+      <c r="F82" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="G82" s="5"/>
+      <c r="G82" s="6"/>
       <c r="H82" s="2" t="s">
         <v>345</v>
       </c>
@@ -4010,10 +4010,10 @@
       </c>
     </row>
     <row r="83" spans="1:9" ht="18" customHeight="1">
-      <c r="A83" s="6" t="s">
+      <c r="A83" s="4" t="s">
         <v>347</v>
       </c>
-      <c r="B83" s="4" t="s">
+      <c r="B83" s="5" t="s">
         <v>348</v>
       </c>
       <c r="C83" s="3" t="s">
@@ -4025,10 +4025,10 @@
       <c r="E83" s="3">
         <v>164</v>
       </c>
-      <c r="F83" s="5" t="s">
+      <c r="F83" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="G83" s="5"/>
+      <c r="G83" s="6"/>
       <c r="H83" s="2" t="s">
         <v>351</v>
       </c>
@@ -4037,8 +4037,8 @@
       </c>
     </row>
     <row r="84" spans="1:9" ht="18" customHeight="1">
-      <c r="A84" s="6"/>
-      <c r="B84" s="4"/>
+      <c r="A84" s="4"/>
+      <c r="B84" s="5"/>
       <c r="C84" s="3" t="s">
         <v>353</v>
       </c>
@@ -4048,10 +4048,10 @@
       <c r="E84" s="3">
         <v>166</v>
       </c>
-      <c r="F84" s="5" t="s">
+      <c r="F84" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="G84" s="5"/>
+      <c r="G84" s="6"/>
       <c r="H84" s="2" t="s">
         <v>355</v>
       </c>
@@ -4060,8 +4060,8 @@
       </c>
     </row>
     <row r="85" spans="1:9" ht="18" customHeight="1">
-      <c r="A85" s="6"/>
-      <c r="B85" s="4"/>
+      <c r="A85" s="4"/>
+      <c r="B85" s="5"/>
       <c r="C85" s="3" t="s">
         <v>357</v>
       </c>
@@ -4071,10 +4071,10 @@
       <c r="E85" s="3">
         <v>168</v>
       </c>
-      <c r="F85" s="5" t="s">
+      <c r="F85" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="G85" s="5"/>
+      <c r="G85" s="6"/>
       <c r="H85" s="2" t="s">
         <v>359</v>
       </c>
@@ -4083,8 +4083,8 @@
       </c>
     </row>
     <row r="86" spans="1:9" ht="18" customHeight="1">
-      <c r="A86" s="6"/>
-      <c r="B86" s="4"/>
+      <c r="A86" s="4"/>
+      <c r="B86" s="5"/>
       <c r="C86" s="3" t="s">
         <v>361</v>
       </c>
@@ -4094,10 +4094,10 @@
       <c r="E86" s="3">
         <v>170</v>
       </c>
-      <c r="F86" s="5" t="s">
+      <c r="F86" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="G86" s="5"/>
+      <c r="G86" s="6"/>
       <c r="H86" s="2" t="s">
         <v>363</v>
       </c>
@@ -4106,8 +4106,8 @@
       </c>
     </row>
     <row r="87" spans="1:9" ht="18" customHeight="1">
-      <c r="A87" s="6"/>
-      <c r="B87" s="4"/>
+      <c r="A87" s="4"/>
+      <c r="B87" s="5"/>
       <c r="C87" s="3" t="s">
         <v>365</v>
       </c>
@@ -4117,10 +4117,10 @@
       <c r="E87" s="3">
         <v>172</v>
       </c>
-      <c r="F87" s="5" t="s">
+      <c r="F87" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="G87" s="5"/>
+      <c r="G87" s="6"/>
       <c r="H87" s="2" t="s">
         <v>367</v>
       </c>
@@ -4129,8 +4129,8 @@
       </c>
     </row>
     <row r="88" spans="1:9" ht="18" customHeight="1">
-      <c r="A88" s="6"/>
-      <c r="B88" s="4"/>
+      <c r="A88" s="4"/>
+      <c r="B88" s="5"/>
       <c r="C88" s="3" t="s">
         <v>369</v>
       </c>
@@ -4140,10 +4140,10 @@
       <c r="E88" s="3">
         <v>174</v>
       </c>
-      <c r="F88" s="5" t="s">
+      <c r="F88" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="G88" s="5"/>
+      <c r="G88" s="6"/>
       <c r="H88" s="2" t="s">
         <v>371</v>
       </c>
@@ -4152,10 +4152,10 @@
       </c>
     </row>
     <row r="89" spans="1:9" ht="18" customHeight="1">
-      <c r="A89" s="6" t="s">
+      <c r="A89" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="B89" s="4" t="s">
+      <c r="B89" s="5" t="s">
         <v>374</v>
       </c>
       <c r="C89" s="3" t="s">
@@ -4167,10 +4167,10 @@
       <c r="E89" s="3">
         <v>176</v>
       </c>
-      <c r="F89" s="5" t="s">
+      <c r="F89" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="G89" s="5"/>
+      <c r="G89" s="6"/>
       <c r="H89" s="2" t="s">
         <v>377</v>
       </c>
@@ -4179,8 +4179,8 @@
       </c>
     </row>
     <row r="90" spans="1:9" ht="18" customHeight="1">
-      <c r="A90" s="6"/>
-      <c r="B90" s="4"/>
+      <c r="A90" s="4"/>
+      <c r="B90" s="5"/>
       <c r="C90" s="3" t="s">
         <v>379</v>
       </c>
@@ -4190,10 +4190,10 @@
       <c r="E90" s="3">
         <v>178</v>
       </c>
-      <c r="F90" s="5" t="s">
+      <c r="F90" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="G90" s="5"/>
+      <c r="G90" s="6"/>
       <c r="H90" s="2" t="s">
         <v>381</v>
       </c>
@@ -4202,8 +4202,8 @@
       </c>
     </row>
     <row r="91" spans="1:9" ht="18" customHeight="1">
-      <c r="A91" s="6"/>
-      <c r="B91" s="4"/>
+      <c r="A91" s="4"/>
+      <c r="B91" s="5"/>
       <c r="C91" s="3" t="s">
         <v>383</v>
       </c>
@@ -4213,10 +4213,10 @@
       <c r="E91" s="3">
         <v>180</v>
       </c>
-      <c r="F91" s="5" t="s">
+      <c r="F91" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="G91" s="5"/>
+      <c r="G91" s="6"/>
       <c r="H91" s="2" t="s">
         <v>385</v>
       </c>
@@ -4225,8 +4225,8 @@
       </c>
     </row>
     <row r="92" spans="1:9" ht="18" customHeight="1">
-      <c r="A92" s="6"/>
-      <c r="B92" s="4"/>
+      <c r="A92" s="4"/>
+      <c r="B92" s="5"/>
       <c r="C92" s="3" t="s">
         <v>387</v>
       </c>
@@ -4236,10 +4236,10 @@
       <c r="E92" s="3">
         <v>182</v>
       </c>
-      <c r="F92" s="5" t="s">
+      <c r="F92" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="G92" s="5"/>
+      <c r="G92" s="6"/>
       <c r="H92" s="2" t="s">
         <v>389</v>
       </c>
@@ -4248,8 +4248,8 @@
       </c>
     </row>
     <row r="93" spans="1:9" ht="18" customHeight="1">
-      <c r="A93" s="6"/>
-      <c r="B93" s="4"/>
+      <c r="A93" s="4"/>
+      <c r="B93" s="5"/>
       <c r="C93" s="3" t="s">
         <v>391</v>
       </c>
@@ -4259,10 +4259,10 @@
       <c r="E93" s="3">
         <v>184</v>
       </c>
-      <c r="F93" s="5" t="s">
+      <c r="F93" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="G93" s="5"/>
+      <c r="G93" s="6"/>
       <c r="H93" s="2" t="s">
         <v>393</v>
       </c>
@@ -4271,8 +4271,8 @@
       </c>
     </row>
     <row r="94" spans="1:9" ht="18" customHeight="1">
-      <c r="A94" s="6"/>
-      <c r="B94" s="4"/>
+      <c r="A94" s="4"/>
+      <c r="B94" s="5"/>
       <c r="C94" s="3" t="s">
         <v>395</v>
       </c>
@@ -4282,10 +4282,10 @@
       <c r="E94" s="3">
         <v>186</v>
       </c>
-      <c r="F94" s="5" t="s">
+      <c r="F94" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="G94" s="5"/>
+      <c r="G94" s="6"/>
       <c r="H94" s="2" t="s">
         <v>397</v>
       </c>
@@ -4294,8 +4294,8 @@
       </c>
     </row>
     <row r="95" spans="1:9" ht="18" customHeight="1">
-      <c r="A95" s="6"/>
-      <c r="B95" s="4"/>
+      <c r="A95" s="4"/>
+      <c r="B95" s="5"/>
       <c r="C95" s="3" t="s">
         <v>399</v>
       </c>
@@ -4305,10 +4305,10 @@
       <c r="E95" s="3">
         <v>188</v>
       </c>
-      <c r="F95" s="5" t="s">
+      <c r="F95" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="G95" s="5"/>
+      <c r="G95" s="6"/>
       <c r="H95" s="2" t="s">
         <v>401</v>
       </c>
@@ -4317,10 +4317,10 @@
       </c>
     </row>
     <row r="96" spans="1:9" ht="18" customHeight="1">
-      <c r="A96" s="6" t="s">
+      <c r="A96" s="4" t="s">
         <v>403</v>
       </c>
-      <c r="B96" s="4" t="s">
+      <c r="B96" s="5" t="s">
         <v>526</v>
       </c>
       <c r="C96" s="3" t="s">
@@ -4332,10 +4332,10 @@
       <c r="E96" s="3">
         <v>190</v>
       </c>
-      <c r="F96" s="5" t="s">
+      <c r="F96" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="G96" s="5"/>
+      <c r="G96" s="6"/>
       <c r="H96" s="2" t="s">
         <v>406</v>
       </c>
@@ -4344,8 +4344,8 @@
       </c>
     </row>
     <row r="97" spans="1:9" ht="18" customHeight="1">
-      <c r="A97" s="6"/>
-      <c r="B97" s="4"/>
+      <c r="A97" s="4"/>
+      <c r="B97" s="5"/>
       <c r="C97" s="3" t="s">
         <v>408</v>
       </c>
@@ -4355,10 +4355,10 @@
       <c r="E97" s="3">
         <v>192</v>
       </c>
-      <c r="F97" s="5" t="s">
+      <c r="F97" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="G97" s="5"/>
+      <c r="G97" s="6"/>
       <c r="H97" s="2" t="s">
         <v>410</v>
       </c>
@@ -4367,8 +4367,8 @@
       </c>
     </row>
     <row r="98" spans="1:9" ht="18" customHeight="1">
-      <c r="A98" s="6"/>
-      <c r="B98" s="4"/>
+      <c r="A98" s="4"/>
+      <c r="B98" s="5"/>
       <c r="C98" s="3" t="s">
         <v>412</v>
       </c>
@@ -4378,10 +4378,10 @@
       <c r="E98" s="3">
         <v>194</v>
       </c>
-      <c r="F98" s="5" t="s">
+      <c r="F98" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="G98" s="5"/>
+      <c r="G98" s="6"/>
       <c r="H98" s="2" t="s">
         <v>414</v>
       </c>
@@ -4390,8 +4390,8 @@
       </c>
     </row>
     <row r="99" spans="1:9" ht="18" customHeight="1">
-      <c r="A99" s="6"/>
-      <c r="B99" s="4"/>
+      <c r="A99" s="4"/>
+      <c r="B99" s="5"/>
       <c r="C99" s="3" t="s">
         <v>416</v>
       </c>
@@ -4401,10 +4401,10 @@
       <c r="E99" s="3">
         <v>196</v>
       </c>
-      <c r="F99" s="5" t="s">
+      <c r="F99" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="G99" s="5"/>
+      <c r="G99" s="6"/>
       <c r="H99" s="2" t="s">
         <v>418</v>
       </c>
@@ -4413,8 +4413,8 @@
       </c>
     </row>
     <row r="100" spans="1:9" ht="18" customHeight="1">
-      <c r="A100" s="6"/>
-      <c r="B100" s="4"/>
+      <c r="A100" s="4"/>
+      <c r="B100" s="5"/>
       <c r="C100" s="3" t="s">
         <v>420</v>
       </c>
@@ -4424,10 +4424,10 @@
       <c r="E100" s="3">
         <v>198</v>
       </c>
-      <c r="F100" s="5" t="s">
+      <c r="F100" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="G100" s="5"/>
+      <c r="G100" s="6"/>
       <c r="H100" s="2" t="s">
         <v>422</v>
       </c>
@@ -4436,8 +4436,8 @@
       </c>
     </row>
     <row r="101" spans="1:9" ht="18" customHeight="1">
-      <c r="A101" s="6"/>
-      <c r="B101" s="4" t="s">
+      <c r="A101" s="4"/>
+      <c r="B101" s="5" t="s">
         <v>424</v>
       </c>
       <c r="C101" s="3" t="s">
@@ -4449,10 +4449,10 @@
       <c r="E101" s="3">
         <v>200</v>
       </c>
-      <c r="F101" s="5" t="s">
+      <c r="F101" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="G101" s="5"/>
+      <c r="G101" s="6"/>
       <c r="H101" s="2" t="s">
         <v>427</v>
       </c>
@@ -4461,8 +4461,8 @@
       </c>
     </row>
     <row r="102" spans="1:9" ht="18" customHeight="1">
-      <c r="A102" s="6"/>
-      <c r="B102" s="4"/>
+      <c r="A102" s="4"/>
+      <c r="B102" s="5"/>
       <c r="C102" s="3" t="s">
         <v>429</v>
       </c>
@@ -4472,10 +4472,10 @@
       <c r="E102" s="3">
         <v>202</v>
       </c>
-      <c r="F102" s="5" t="s">
+      <c r="F102" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="G102" s="5"/>
+      <c r="G102" s="6"/>
       <c r="H102" s="2" t="s">
         <v>431</v>
       </c>
@@ -4484,8 +4484,8 @@
       </c>
     </row>
     <row r="103" spans="1:9" ht="18" customHeight="1">
-      <c r="A103" s="6"/>
-      <c r="B103" s="4"/>
+      <c r="A103" s="4"/>
+      <c r="B103" s="5"/>
       <c r="C103" s="3" t="s">
         <v>433</v>
       </c>
@@ -4495,10 +4495,10 @@
       <c r="E103" s="3">
         <v>204</v>
       </c>
-      <c r="F103" s="5" t="s">
+      <c r="F103" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="G103" s="5"/>
+      <c r="G103" s="6"/>
       <c r="H103" s="2" t="s">
         <v>435</v>
       </c>
@@ -4507,8 +4507,8 @@
       </c>
     </row>
     <row r="104" spans="1:9" ht="18" customHeight="1">
-      <c r="A104" s="6"/>
-      <c r="B104" s="4"/>
+      <c r="A104" s="4"/>
+      <c r="B104" s="5"/>
       <c r="C104" s="3" t="s">
         <v>437</v>
       </c>
@@ -4518,10 +4518,10 @@
       <c r="E104" s="3">
         <v>206</v>
       </c>
-      <c r="F104" s="5" t="s">
+      <c r="F104" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="G104" s="5"/>
+      <c r="G104" s="6"/>
       <c r="H104" s="2" t="s">
         <v>439</v>
       </c>
@@ -4530,8 +4530,8 @@
       </c>
     </row>
     <row r="105" spans="1:9" ht="18" customHeight="1">
-      <c r="A105" s="6"/>
-      <c r="B105" s="4"/>
+      <c r="A105" s="4"/>
+      <c r="B105" s="5"/>
       <c r="C105" s="3" t="s">
         <v>441</v>
       </c>
@@ -4541,10 +4541,10 @@
       <c r="E105" s="3">
         <v>208</v>
       </c>
-      <c r="F105" s="5" t="s">
+      <c r="F105" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="G105" s="5"/>
+      <c r="G105" s="6"/>
       <c r="H105" s="2" t="s">
         <v>443</v>
       </c>
@@ -4553,8 +4553,8 @@
       </c>
     </row>
     <row r="106" spans="1:9" ht="18" customHeight="1">
-      <c r="A106" s="6"/>
-      <c r="B106" s="4"/>
+      <c r="A106" s="4"/>
+      <c r="B106" s="5"/>
       <c r="C106" s="3" t="s">
         <v>445</v>
       </c>
@@ -4564,10 +4564,10 @@
       <c r="E106" s="3">
         <v>210</v>
       </c>
-      <c r="F106" s="5" t="s">
+      <c r="F106" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="G106" s="5"/>
+      <c r="G106" s="6"/>
       <c r="H106" s="2" t="s">
         <v>447</v>
       </c>
@@ -4576,10 +4576,10 @@
       </c>
     </row>
     <row r="107" spans="1:9" ht="18" customHeight="1">
-      <c r="A107" s="6" t="s">
+      <c r="A107" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="B107" s="4" t="s">
+      <c r="B107" s="5" t="s">
         <v>450</v>
       </c>
       <c r="C107" s="3" t="s">
@@ -4591,10 +4591,10 @@
       <c r="E107" s="3">
         <v>212</v>
       </c>
-      <c r="F107" s="5" t="s">
+      <c r="F107" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="G107" s="5"/>
+      <c r="G107" s="6"/>
       <c r="H107" s="2" t="s">
         <v>453</v>
       </c>
@@ -4603,8 +4603,8 @@
       </c>
     </row>
     <row r="108" spans="1:9" ht="18" customHeight="1">
-      <c r="A108" s="6"/>
-      <c r="B108" s="4"/>
+      <c r="A108" s="4"/>
+      <c r="B108" s="5"/>
       <c r="C108" s="3" t="s">
         <v>455</v>
       </c>
@@ -4614,10 +4614,10 @@
       <c r="E108" s="3">
         <v>214</v>
       </c>
-      <c r="F108" s="5" t="s">
+      <c r="F108" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="G108" s="5"/>
+      <c r="G108" s="6"/>
       <c r="H108" s="2" t="s">
         <v>457</v>
       </c>
@@ -4626,8 +4626,8 @@
       </c>
     </row>
     <row r="109" spans="1:9" ht="18" customHeight="1">
-      <c r="A109" s="6"/>
-      <c r="B109" s="4" t="s">
+      <c r="A109" s="4"/>
+      <c r="B109" s="5" t="s">
         <v>459</v>
       </c>
       <c r="C109" s="3" t="s">
@@ -4639,10 +4639,10 @@
       <c r="E109" s="3">
         <v>216</v>
       </c>
-      <c r="F109" s="5" t="s">
+      <c r="F109" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="G109" s="5"/>
+      <c r="G109" s="6"/>
       <c r="H109" s="2" t="s">
         <v>462</v>
       </c>
@@ -4651,8 +4651,8 @@
       </c>
     </row>
     <row r="110" spans="1:9" ht="18" customHeight="1">
-      <c r="A110" s="6"/>
-      <c r="B110" s="4"/>
+      <c r="A110" s="4"/>
+      <c r="B110" s="5"/>
       <c r="C110" s="3" t="s">
         <v>464</v>
       </c>
@@ -4662,10 +4662,10 @@
       <c r="E110" s="3">
         <v>218</v>
       </c>
-      <c r="F110" s="5" t="s">
+      <c r="F110" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="G110" s="5"/>
+      <c r="G110" s="6"/>
       <c r="H110" s="2" t="s">
         <v>466</v>
       </c>
@@ -4674,8 +4674,8 @@
       </c>
     </row>
     <row r="111" spans="1:9" ht="18" customHeight="1">
-      <c r="A111" s="6"/>
-      <c r="B111" s="4" t="s">
+      <c r="A111" s="4"/>
+      <c r="B111" s="5" t="s">
         <v>468</v>
       </c>
       <c r="C111" s="3" t="s">
@@ -4687,10 +4687,10 @@
       <c r="E111" s="3">
         <v>220</v>
       </c>
-      <c r="F111" s="5" t="s">
+      <c r="F111" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="G111" s="5"/>
+      <c r="G111" s="6"/>
       <c r="H111" s="2" t="s">
         <v>471</v>
       </c>
@@ -4699,8 +4699,8 @@
       </c>
     </row>
     <row r="112" spans="1:9" ht="18" customHeight="1">
-      <c r="A112" s="6"/>
-      <c r="B112" s="4"/>
+      <c r="A112" s="4"/>
+      <c r="B112" s="5"/>
       <c r="C112" s="3" t="s">
         <v>473</v>
       </c>
@@ -4710,10 +4710,10 @@
       <c r="E112" s="3">
         <v>222</v>
       </c>
-      <c r="F112" s="5" t="s">
+      <c r="F112" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="G112" s="5"/>
+      <c r="G112" s="6"/>
       <c r="H112" s="2" t="s">
         <v>475</v>
       </c>
@@ -4722,8 +4722,8 @@
       </c>
     </row>
     <row r="113" spans="1:9" ht="18" customHeight="1">
-      <c r="A113" s="6"/>
-      <c r="B113" s="4"/>
+      <c r="A113" s="4"/>
+      <c r="B113" s="5"/>
       <c r="C113" s="3" t="s">
         <v>477</v>
       </c>
@@ -4733,10 +4733,10 @@
       <c r="E113" s="3">
         <v>224</v>
       </c>
-      <c r="F113" s="5" t="s">
+      <c r="F113" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="G113" s="5"/>
+      <c r="G113" s="6"/>
       <c r="H113" s="2" t="s">
         <v>479</v>
       </c>
@@ -4745,8 +4745,8 @@
       </c>
     </row>
     <row r="114" spans="1:9" ht="18" customHeight="1">
-      <c r="A114" s="6"/>
-      <c r="B114" s="4"/>
+      <c r="A114" s="4"/>
+      <c r="B114" s="5"/>
       <c r="C114" s="3" t="s">
         <v>481</v>
       </c>
@@ -4756,10 +4756,10 @@
       <c r="E114" s="3">
         <v>226</v>
       </c>
-      <c r="F114" s="5" t="s">
+      <c r="F114" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="G114" s="5"/>
+      <c r="G114" s="6"/>
       <c r="H114" s="2" t="s">
         <v>483</v>
       </c>
@@ -4768,8 +4768,8 @@
       </c>
     </row>
     <row r="115" spans="1:9" ht="18" customHeight="1">
-      <c r="A115" s="6"/>
-      <c r="B115" s="4"/>
+      <c r="A115" s="4"/>
+      <c r="B115" s="5"/>
       <c r="C115" s="3" t="s">
         <v>485</v>
       </c>
@@ -4779,10 +4779,10 @@
       <c r="E115" s="3">
         <v>228</v>
       </c>
-      <c r="F115" s="5" t="s">
+      <c r="F115" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="G115" s="5"/>
+      <c r="G115" s="6"/>
       <c r="H115" s="2" t="s">
         <v>487</v>
       </c>
@@ -4791,8 +4791,8 @@
       </c>
     </row>
     <row r="116" spans="1:9" ht="18" customHeight="1">
-      <c r="A116" s="6"/>
-      <c r="B116" s="4"/>
+      <c r="A116" s="4"/>
+      <c r="B116" s="5"/>
       <c r="C116" s="3" t="s">
         <v>489</v>
       </c>
@@ -4802,10 +4802,10 @@
       <c r="E116" s="3">
         <v>230</v>
       </c>
-      <c r="F116" s="5" t="s">
+      <c r="F116" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="G116" s="5"/>
+      <c r="G116" s="6"/>
       <c r="H116" s="2" t="s">
         <v>491</v>
       </c>
@@ -4814,8 +4814,8 @@
       </c>
     </row>
     <row r="117" spans="1:9" ht="18" customHeight="1">
-      <c r="A117" s="6"/>
-      <c r="B117" s="4" t="s">
+      <c r="A117" s="4"/>
+      <c r="B117" s="5" t="s">
         <v>493</v>
       </c>
       <c r="C117" s="3" t="s">
@@ -4827,10 +4827,10 @@
       <c r="E117" s="3">
         <v>232</v>
       </c>
-      <c r="F117" s="5" t="s">
+      <c r="F117" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="G117" s="5"/>
+      <c r="G117" s="6"/>
       <c r="H117" s="2" t="s">
         <v>496</v>
       </c>
@@ -4839,8 +4839,8 @@
       </c>
     </row>
     <row r="118" spans="1:9" ht="18" customHeight="1">
-      <c r="A118" s="6"/>
-      <c r="B118" s="4"/>
+      <c r="A118" s="4"/>
+      <c r="B118" s="5"/>
       <c r="C118" s="3" t="s">
         <v>498</v>
       </c>
@@ -4850,10 +4850,10 @@
       <c r="E118" s="3">
         <v>234</v>
       </c>
-      <c r="F118" s="5" t="s">
+      <c r="F118" s="6" t="s">
         <v>499</v>
       </c>
-      <c r="G118" s="5"/>
+      <c r="G118" s="6"/>
       <c r="H118" s="2" t="s">
         <v>500</v>
       </c>
@@ -4862,8 +4862,8 @@
       </c>
     </row>
     <row r="119" spans="1:9" ht="18" customHeight="1">
-      <c r="A119" s="6"/>
-      <c r="B119" s="4"/>
+      <c r="A119" s="4"/>
+      <c r="B119" s="5"/>
       <c r="C119" s="3" t="s">
         <v>502</v>
       </c>
@@ -4873,10 +4873,10 @@
       <c r="E119" s="3">
         <v>236</v>
       </c>
-      <c r="F119" s="5" t="s">
+      <c r="F119" s="6" t="s">
         <v>503</v>
       </c>
-      <c r="G119" s="5"/>
+      <c r="G119" s="6"/>
       <c r="H119" s="2" t="s">
         <v>504</v>
       </c>
@@ -4885,8 +4885,8 @@
       </c>
     </row>
     <row r="120" spans="1:9" ht="18" customHeight="1">
-      <c r="A120" s="6"/>
-      <c r="B120" s="4"/>
+      <c r="A120" s="4"/>
+      <c r="B120" s="5"/>
       <c r="C120" s="3" t="s">
         <v>506</v>
       </c>
@@ -4896,10 +4896,10 @@
       <c r="E120" s="3">
         <v>238</v>
       </c>
-      <c r="F120" s="5" t="s">
+      <c r="F120" s="6" t="s">
         <v>507</v>
       </c>
-      <c r="G120" s="5"/>
+      <c r="G120" s="6"/>
       <c r="H120" s="2" t="s">
         <v>508</v>
       </c>
@@ -4908,8 +4908,8 @@
       </c>
     </row>
     <row r="121" spans="1:9" ht="18" customHeight="1">
-      <c r="A121" s="6"/>
-      <c r="B121" s="4"/>
+      <c r="A121" s="4"/>
+      <c r="B121" s="5"/>
       <c r="C121" s="3" t="s">
         <v>510</v>
       </c>
@@ -4919,10 +4919,10 @@
       <c r="E121" s="3">
         <v>240</v>
       </c>
-      <c r="F121" s="5" t="s">
+      <c r="F121" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="G121" s="5"/>
+      <c r="G121" s="6"/>
       <c r="H121" s="2" t="s">
         <v>512</v>
       </c>
@@ -4931,8 +4931,8 @@
       </c>
     </row>
     <row r="122" spans="1:9" ht="18" customHeight="1">
-      <c r="A122" s="6"/>
-      <c r="B122" s="4"/>
+      <c r="A122" s="4"/>
+      <c r="B122" s="5"/>
       <c r="C122" s="3" t="s">
         <v>514</v>
       </c>
@@ -4942,10 +4942,10 @@
       <c r="E122" s="3">
         <v>242</v>
       </c>
-      <c r="F122" s="5" t="s">
+      <c r="F122" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="G122" s="5"/>
+      <c r="G122" s="6"/>
       <c r="H122" s="2" t="s">
         <v>516</v>
       </c>
@@ -4954,8 +4954,8 @@
       </c>
     </row>
     <row r="123" spans="1:9" ht="18" customHeight="1">
-      <c r="A123" s="6"/>
-      <c r="B123" s="4"/>
+      <c r="A123" s="4"/>
+      <c r="B123" s="5"/>
       <c r="C123" s="3" t="s">
         <v>518</v>
       </c>
@@ -4965,10 +4965,10 @@
       <c r="E123" s="3">
         <v>244</v>
       </c>
-      <c r="F123" s="5" t="s">
+      <c r="F123" s="6" t="s">
         <v>519</v>
       </c>
-      <c r="G123" s="5"/>
+      <c r="G123" s="6"/>
       <c r="H123" s="2" t="s">
         <v>520</v>
       </c>
@@ -4977,8 +4977,8 @@
       </c>
     </row>
     <row r="124" spans="1:9" ht="18" customHeight="1">
-      <c r="A124" s="6"/>
-      <c r="B124" s="4"/>
+      <c r="A124" s="4"/>
+      <c r="B124" s="5"/>
       <c r="C124" s="3" t="s">
         <v>522</v>
       </c>
@@ -4988,10 +4988,10 @@
       <c r="E124" s="3">
         <v>246</v>
       </c>
-      <c r="F124" s="5" t="s">
+      <c r="F124" s="6" t="s">
         <v>523</v>
       </c>
-      <c r="G124" s="5"/>
+      <c r="G124" s="6"/>
       <c r="H124" s="2" t="s">
         <v>524</v>
       </c>
@@ -5001,6 +5001,137 @@
     </row>
   </sheetData>
   <mergeCells count="155">
+    <mergeCell ref="F103:G103"/>
+    <mergeCell ref="F104:G104"/>
+    <mergeCell ref="F105:G105"/>
+    <mergeCell ref="F106:G106"/>
+    <mergeCell ref="B117:B124"/>
+    <mergeCell ref="F117:G117"/>
+    <mergeCell ref="F118:G118"/>
+    <mergeCell ref="F119:G119"/>
+    <mergeCell ref="F120:G120"/>
+    <mergeCell ref="F121:G121"/>
+    <mergeCell ref="F122:G122"/>
+    <mergeCell ref="F123:G123"/>
+    <mergeCell ref="F124:G124"/>
+    <mergeCell ref="A107:A124"/>
+    <mergeCell ref="B107:B108"/>
+    <mergeCell ref="F107:G107"/>
+    <mergeCell ref="F108:G108"/>
+    <mergeCell ref="B109:B110"/>
+    <mergeCell ref="F109:G109"/>
+    <mergeCell ref="A96:A106"/>
+    <mergeCell ref="B96:B100"/>
+    <mergeCell ref="F96:G96"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="F98:G98"/>
+    <mergeCell ref="F99:G99"/>
+    <mergeCell ref="F100:G100"/>
+    <mergeCell ref="B101:B106"/>
+    <mergeCell ref="F101:G101"/>
+    <mergeCell ref="F102:G102"/>
+    <mergeCell ref="F110:G110"/>
+    <mergeCell ref="B111:B116"/>
+    <mergeCell ref="F111:G111"/>
+    <mergeCell ref="F112:G112"/>
+    <mergeCell ref="F113:G113"/>
+    <mergeCell ref="F114:G114"/>
+    <mergeCell ref="F115:G115"/>
+    <mergeCell ref="F116:G116"/>
+    <mergeCell ref="A89:A95"/>
+    <mergeCell ref="B89:B95"/>
+    <mergeCell ref="F89:G89"/>
+    <mergeCell ref="F90:G90"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="F92:G92"/>
+    <mergeCell ref="F93:G93"/>
+    <mergeCell ref="F94:G94"/>
+    <mergeCell ref="F95:G95"/>
+    <mergeCell ref="A83:A88"/>
+    <mergeCell ref="B83:B88"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="F85:G85"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="F87:G87"/>
+    <mergeCell ref="F88:G88"/>
+    <mergeCell ref="B75:B78"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="B79:B82"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="A64:A82"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="B69:B74"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="B62:B63"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="B64:B68"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="B53:B55"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="B56:B61"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="A36:A63"/>
+    <mergeCell ref="B36:B41"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="F38:G38"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="F40:G40"/>
+    <mergeCell ref="B46:B52"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="F49:G49"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="B28:B33"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B22:B27"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="E1:F1"/>
     <mergeCell ref="A2:A35"/>
     <mergeCell ref="B2:B8"/>
@@ -5025,137 +5156,6 @@
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="F13:G13"/>
     <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="B28:B33"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="B22:B27"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="F23:G23"/>
-    <mergeCell ref="F24:G24"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="A36:A63"/>
-    <mergeCell ref="B36:B41"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="F38:G38"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="B46:B52"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="F49:G49"/>
-    <mergeCell ref="F50:G50"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="B42:B45"/>
-    <mergeCell ref="F42:G42"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="B53:B55"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="B56:B61"/>
-    <mergeCell ref="F56:G56"/>
-    <mergeCell ref="F57:G57"/>
-    <mergeCell ref="F58:G58"/>
-    <mergeCell ref="F59:G59"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="B69:B74"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="B62:B63"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="B64:B68"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="A83:A88"/>
-    <mergeCell ref="B83:B88"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="F86:G86"/>
-    <mergeCell ref="F87:G87"/>
-    <mergeCell ref="F88:G88"/>
-    <mergeCell ref="B75:B78"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="F77:G77"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="B79:B82"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="A64:A82"/>
-    <mergeCell ref="A89:A95"/>
-    <mergeCell ref="B89:B95"/>
-    <mergeCell ref="F89:G89"/>
-    <mergeCell ref="F90:G90"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="F92:G92"/>
-    <mergeCell ref="F93:G93"/>
-    <mergeCell ref="F94:G94"/>
-    <mergeCell ref="F95:G95"/>
-    <mergeCell ref="A107:A124"/>
-    <mergeCell ref="B107:B108"/>
-    <mergeCell ref="F107:G107"/>
-    <mergeCell ref="F108:G108"/>
-    <mergeCell ref="B109:B110"/>
-    <mergeCell ref="F109:G109"/>
-    <mergeCell ref="A96:A106"/>
-    <mergeCell ref="B96:B100"/>
-    <mergeCell ref="F96:G96"/>
-    <mergeCell ref="F97:G97"/>
-    <mergeCell ref="F98:G98"/>
-    <mergeCell ref="F99:G99"/>
-    <mergeCell ref="F100:G100"/>
-    <mergeCell ref="B101:B106"/>
-    <mergeCell ref="F101:G101"/>
-    <mergeCell ref="F102:G102"/>
-    <mergeCell ref="F110:G110"/>
-    <mergeCell ref="B111:B116"/>
-    <mergeCell ref="F111:G111"/>
-    <mergeCell ref="F112:G112"/>
-    <mergeCell ref="F113:G113"/>
-    <mergeCell ref="F114:G114"/>
-    <mergeCell ref="F115:G115"/>
-    <mergeCell ref="F116:G116"/>
-    <mergeCell ref="F103:G103"/>
-    <mergeCell ref="F104:G104"/>
-    <mergeCell ref="F105:G105"/>
-    <mergeCell ref="F106:G106"/>
-    <mergeCell ref="B117:B124"/>
-    <mergeCell ref="F117:G117"/>
-    <mergeCell ref="F118:G118"/>
-    <mergeCell ref="F119:G119"/>
-    <mergeCell ref="F120:G120"/>
-    <mergeCell ref="F121:G121"/>
-    <mergeCell ref="F122:G122"/>
-    <mergeCell ref="F123:G123"/>
-    <mergeCell ref="F124:G124"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>